<commit_message>
add data on soil sorption and degradation
for Propamocarb, Halauxifen-methyl and Ferric phosphate
</commit_message>
<xml_diff>
--- a/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
+++ b/data_generation/06_soil_sorption/acetamiprid_soil_sorption.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\06_soil_sorption\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DF5A32-7623-48E5-AF73-E7F8AA07D377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499BFB4A-F8A4-44C0-8185-98A378FB8050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="410" yWindow="520" windowWidth="28800" windowHeight="15410" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2660" windowWidth="19380" windowHeight="5620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="40">
   <si>
     <t>soil_type</t>
   </si>
@@ -133,6 +133,18 @@
   </si>
   <si>
     <t>Kfoc</t>
+  </si>
+  <si>
+    <t>one_over_n</t>
+  </si>
+  <si>
+    <t>mean</t>
+  </si>
+  <si>
+    <t>mean_type</t>
+  </si>
+  <si>
+    <t>FALSE</t>
   </si>
 </sst>
 </file>
@@ -176,10 +188,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,16 +534,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="23.26953125" customWidth="1"/>
     <col min="3" max="3" width="19.26953125" customWidth="1"/>
     <col min="5" max="5" width="12.7265625" customWidth="1"/>
-    <col min="16" max="16" width="45.1796875" customWidth="1"/>
+    <col min="19" max="19" width="45.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" s="1" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -571,32 +586,41 @@
       <c r="N1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -622,22 +646,25 @@
         <v>0.84199999999999997</v>
       </c>
       <c r="P2" t="s">
+        <v>39</v>
+      </c>
+      <c r="S2" t="s">
         <v>14</v>
       </c>
-      <c r="Q2">
+      <c r="T2">
         <v>32</v>
       </c>
-      <c r="R2" t="s">
+      <c r="U2" t="s">
         <v>13</v>
       </c>
-      <c r="S2" t="s">
+      <c r="V2" t="s">
         <v>9</v>
       </c>
-      <c r="U2" t="s">
+      <c r="X2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -663,22 +690,25 @@
         <v>0.82499999999999996</v>
       </c>
       <c r="P3" t="s">
+        <v>39</v>
+      </c>
+      <c r="S3" t="s">
         <v>14</v>
       </c>
-      <c r="Q3">
+      <c r="T3">
         <v>32</v>
       </c>
-      <c r="R3" t="s">
+      <c r="U3" t="s">
         <v>13</v>
       </c>
-      <c r="S3" t="s">
+      <c r="V3" t="s">
         <v>9</v>
       </c>
-      <c r="U3" t="s">
+      <c r="X3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -704,22 +734,25 @@
         <v>0.89300000000000002</v>
       </c>
       <c r="P4" t="s">
+        <v>39</v>
+      </c>
+      <c r="S4" t="s">
         <v>14</v>
       </c>
-      <c r="Q4">
+      <c r="T4">
         <v>32</v>
       </c>
-      <c r="R4" t="s">
+      <c r="U4" t="s">
         <v>13</v>
       </c>
-      <c r="S4" t="s">
+      <c r="V4" t="s">
         <v>9</v>
       </c>
-      <c r="U4" t="s">
+      <c r="X4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -745,22 +778,25 @@
         <v>0.83499999999999996</v>
       </c>
       <c r="P5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S5" t="s">
         <v>14</v>
       </c>
-      <c r="Q5">
+      <c r="T5">
         <v>32</v>
       </c>
-      <c r="R5" t="s">
+      <c r="U5" t="s">
         <v>13</v>
       </c>
-      <c r="S5" t="s">
+      <c r="V5" t="s">
         <v>9</v>
       </c>
-      <c r="U5" t="s">
+      <c r="X5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -786,23 +822,26 @@
         <v>0.90700000000000003</v>
       </c>
       <c r="P6" t="s">
+        <v>39</v>
+      </c>
+      <c r="S6" t="s">
         <v>14</v>
       </c>
-      <c r="Q6">
+      <c r="T6">
         <v>32</v>
       </c>
-      <c r="R6" t="s">
+      <c r="U6" t="s">
         <v>13</v>
       </c>
-      <c r="S6" t="s">
+      <c r="V6" t="s">
         <v>9</v>
       </c>
-      <c r="U6" t="s">
+      <c r="X6" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:V6">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Y6">
     <sortCondition ref="C2:C6"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>